<commit_message>
added checks for expected values of --primer_mix, --study_type, and primer_name
</commit_message>
<xml_diff>
--- a/refseq/refseq_all.xlsx
+++ b/refseq/refseq_all.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\groups.biotech.cdc.gov\groups\Projects\EET_Tick_Surveillance\Research\Lynn\2025\02_12_25_MPAS_create_targets_process\08-13-25_MPASv206_addMakeTargets_dev\v206_dev\refseq\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\groups.biotech.cdc.gov\groups\Projects\EET_Tick_Surveillance\Research\Lynn\2026\01-06-26_pipeline_checks_make_targets\v206_dev\refseq\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D97D9E06-8162-4091-AD5D-40878DC031E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8602A465-E8F1-40F3-BCF3-DD70C2A001AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" activeTab="1" xr2:uid="{34BACE26-3AA6-4971-B237-F23C3D32CC55}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{34BACE26-3AA6-4971-B237-F23C3D32CC55}"/>
   </bookViews>
   <sheets>
     <sheet name="targets" sheetId="1" r:id="rId1"/>
@@ -1540,22 +1540,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{660399C9-9375-49BE-A54F-7E2D1E2F5B06}">
-  <dimension ref="A1:P127"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:P126"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="91.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="49.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="77.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="76.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="13" width="15.140625" customWidth="1"/>
+    <col min="1" max="1" width="91.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="49.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="77.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="76.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="13" width="15.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>137</v>
       </c>
@@ -1599,7 +1599,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>331</v>
       </c>
@@ -1643,7 +1643,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>330</v>
       </c>
@@ -1687,7 +1687,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>329</v>
       </c>
@@ -1731,7 +1731,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>186</v>
       </c>
@@ -1775,7 +1775,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>182</v>
       </c>
@@ -1819,7 +1819,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>184</v>
       </c>
@@ -1863,7 +1863,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>183</v>
       </c>
@@ -1907,7 +1907,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>337</v>
       </c>
@@ -1951,7 +1951,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>361</v>
       </c>
@@ -1995,7 +1995,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>138</v>
       </c>
@@ -2039,7 +2039,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>139</v>
       </c>
@@ -2083,7 +2083,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>141</v>
       </c>
@@ -2127,7 +2127,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>142</v>
       </c>
@@ -2171,7 +2171,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>140</v>
       </c>
@@ -2215,7 +2215,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>143</v>
       </c>
@@ -2259,7 +2259,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>144</v>
       </c>
@@ -2303,7 +2303,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>145</v>
       </c>
@@ -2347,7 +2347,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>146</v>
       </c>
@@ -2391,7 +2391,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>150</v>
       </c>
@@ -2435,7 +2435,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>222</v>
       </c>
@@ -2479,7 +2479,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>328</v>
       </c>
@@ -2523,7 +2523,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>327</v>
       </c>
@@ -2567,7 +2567,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>326</v>
       </c>
@@ -2611,7 +2611,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>362</v>
       </c>
@@ -2658,7 +2658,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>147</v>
       </c>
@@ -2702,7 +2702,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>148</v>
       </c>
@@ -2746,7 +2746,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>149</v>
       </c>
@@ -2790,7 +2790,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>154</v>
       </c>
@@ -2834,7 +2834,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>153</v>
       </c>
@@ -2878,7 +2878,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>211</v>
       </c>
@@ -2922,7 +2922,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>210</v>
       </c>
@@ -2966,7 +2966,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>151</v>
       </c>
@@ -3010,7 +3010,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>209</v>
       </c>
@@ -3054,7 +3054,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>208</v>
       </c>
@@ -3098,7 +3098,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>152</v>
       </c>
@@ -3142,7 +3142,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>207</v>
       </c>
@@ -3186,7 +3186,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>206</v>
       </c>
@@ -3230,7 +3230,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>155</v>
       </c>
@@ -3274,7 +3274,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>205</v>
       </c>
@@ -3318,7 +3318,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>194</v>
       </c>
@@ -3362,7 +3362,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>156</v>
       </c>
@@ -3406,7 +3406,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>157</v>
       </c>
@@ -3450,7 +3450,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>363</v>
       </c>
@@ -3494,7 +3494,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>158</v>
       </c>
@@ -3538,7 +3538,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>159</v>
       </c>
@@ -3582,7 +3582,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>160</v>
       </c>
@@ -3626,7 +3626,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>161</v>
       </c>
@@ -3670,7 +3670,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>162</v>
       </c>
@@ -3714,7 +3714,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>163</v>
       </c>
@@ -3758,7 +3758,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>204</v>
       </c>
@@ -3802,7 +3802,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>203</v>
       </c>
@@ -3846,7 +3846,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>164</v>
       </c>
@@ -3890,7 +3890,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>202</v>
       </c>
@@ -3934,7 +3934,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>165</v>
       </c>
@@ -3978,7 +3978,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>167</v>
       </c>
@@ -4022,7 +4022,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>168</v>
       </c>
@@ -4066,7 +4066,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="58" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>169</v>
       </c>
@@ -4110,7 +4110,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>201</v>
       </c>
@@ -4154,7 +4154,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="60" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>166</v>
       </c>
@@ -4198,7 +4198,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="61" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A61" s="3" t="s">
         <v>195</v>
       </c>
@@ -4242,7 +4242,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="62" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A62" s="3" t="s">
         <v>196</v>
       </c>
@@ -4286,7 +4286,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="63" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A63" s="3" t="s">
         <v>197</v>
       </c>
@@ -4330,7 +4330,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="64" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A64" s="3" t="s">
         <v>198</v>
       </c>
@@ -4374,7 +4374,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="65" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A65" s="3" t="s">
         <v>199</v>
       </c>
@@ -4418,7 +4418,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="66" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>200</v>
       </c>
@@ -4462,7 +4462,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="67" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>170</v>
       </c>
@@ -4506,7 +4506,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="68" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>171</v>
       </c>
@@ -4550,7 +4550,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="69" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>215</v>
       </c>
@@ -4594,7 +4594,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="70" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>172</v>
       </c>
@@ -4638,7 +4638,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="71" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>173</v>
       </c>
@@ -4682,7 +4682,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="72" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>174</v>
       </c>
@@ -4726,7 +4726,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="73" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>176</v>
       </c>
@@ -4770,7 +4770,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="74" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>175</v>
       </c>
@@ -4814,7 +4814,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="75" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>193</v>
       </c>
@@ -4858,7 +4858,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="76" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>178</v>
       </c>
@@ -4902,7 +4902,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="77" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>177</v>
       </c>
@@ -4946,7 +4946,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="78" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>339</v>
       </c>
@@ -4990,7 +4990,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="79" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>340</v>
       </c>
@@ -5034,7 +5034,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="80" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>341</v>
       </c>
@@ -5078,7 +5078,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="81" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>342</v>
       </c>
@@ -5122,7 +5122,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="82" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>319</v>
       </c>
@@ -5166,7 +5166,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="83" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>320</v>
       </c>
@@ -5210,7 +5210,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="84" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>321</v>
       </c>
@@ -5254,7 +5254,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="85" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>322</v>
       </c>
@@ -5298,7 +5298,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="86" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>323</v>
       </c>
@@ -5342,7 +5342,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="87" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>324</v>
       </c>
@@ -5386,7 +5386,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="88" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>325</v>
       </c>
@@ -5430,7 +5430,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="89" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>179</v>
       </c>
@@ -5474,7 +5474,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="90" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>180</v>
       </c>
@@ -5518,7 +5518,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="91" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>181</v>
       </c>
@@ -5562,7 +5562,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="92" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>216</v>
       </c>
@@ -5606,7 +5606,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="93" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>217</v>
       </c>
@@ -5650,7 +5650,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="94" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>313</v>
       </c>
@@ -5694,7 +5694,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="95" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>314</v>
       </c>
@@ -5738,7 +5738,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="96" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>315</v>
       </c>
@@ -5782,7 +5782,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="97" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>316</v>
       </c>
@@ -5826,7 +5826,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="98" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>317</v>
       </c>
@@ -5870,7 +5870,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="99" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>318</v>
       </c>
@@ -5914,7 +5914,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="100" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>332</v>
       </c>
@@ -5958,7 +5958,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="101" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>304</v>
       </c>
@@ -6002,7 +6002,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="102" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>305</v>
       </c>
@@ -6046,7 +6046,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="103" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>306</v>
       </c>
@@ -6090,7 +6090,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="104" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>307</v>
       </c>
@@ -6134,7 +6134,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="105" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>308</v>
       </c>
@@ -6178,7 +6178,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="106" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>309</v>
       </c>
@@ -6222,7 +6222,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="107" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>310</v>
       </c>
@@ -6266,7 +6266,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="108" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>311</v>
       </c>
@@ -6310,7 +6310,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="109" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>312</v>
       </c>
@@ -6354,7 +6354,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="110" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>192</v>
       </c>
@@ -6398,7 +6398,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="111" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>303</v>
       </c>
@@ -6442,7 +6442,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="112" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>302</v>
       </c>
@@ -6486,7 +6486,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="113" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>355</v>
       </c>
@@ -6530,7 +6530,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="114" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>364</v>
       </c>
@@ -6574,7 +6574,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="115" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>359</v>
       </c>
@@ -6618,30 +6618,30 @@
         <v>360</v>
       </c>
     </row>
-    <row r="117" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="N117" s="2"/>
-    </row>
-    <row r="119" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="N116" s="2"/>
+    </row>
+    <row r="118" spans="1:14" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="C118" s="1"/>
+    </row>
+    <row r="119" spans="1:14" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C119" s="1"/>
     </row>
-    <row r="120" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:14" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C120" s="1"/>
     </row>
-    <row r="121" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:14" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C121" s="1"/>
     </row>
-    <row r="122" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:14" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C122" s="1"/>
-    </row>
-    <row r="123" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="C123" s="1"/>
-      <c r="E123" s="2"/>
-    </row>
-    <row r="126" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="N126" s="2"/>
-    </row>
-    <row r="127" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="C127" s="1"/>
+      <c r="E122" s="2"/>
+    </row>
+    <row r="125" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="N125" s="2"/>
+    </row>
+    <row r="126" spans="1:14" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="C126" s="1"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:N112" xr:uid="{660399C9-9375-49BE-A54F-7E2D1E2F5B06}"/>
@@ -6657,18 +6657,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67470D7A-4C93-4EF4-9DEE-54C9E733D09A}">
   <dimension ref="A1:H9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.1796875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="44" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="39.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="29.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="39.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="29.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>338</v>
       </c>
@@ -6694,7 +6694,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>132</v>
       </c>
@@ -6717,7 +6717,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>132</v>
       </c>
@@ -6740,7 +6740,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>132</v>
       </c>
@@ -6763,7 +6763,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>132</v>
       </c>
@@ -6786,7 +6786,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>124</v>
       </c>
@@ -6809,7 +6809,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>124</v>
       </c>
@@ -6832,7 +6832,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>124</v>
       </c>
@@ -6855,7 +6855,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>124</v>
       </c>

</xml_diff>